<commit_message>
Fix helmet detection accuracy, update run script and cleanup .gitattributes
</commit_message>
<xml_diff>
--- a/detected_numberplates.xlsx
+++ b/detected_numberplates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,6 +780,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>AP13Q 8816</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-13 20:52:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>triple</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>AP13Q 8815</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-13 20:52:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>AP13Q 8815</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-13 20:52:56</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
models and lib update
</commit_message>
<xml_diff>
--- a/detected_numberplates.xlsx
+++ b/detected_numberplates.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,36 +413,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Unnamed: 1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Unnamed: 2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>AlertType</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>NumberPlate</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
@@ -840,6 +828,46 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>AP28 BA 7090</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-04-14 21:09:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>DL 14S C0887</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-04-14 21:33:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>